<commit_message>
vault backup: 2026-10-19 09:52:12
</commit_message>
<xml_diff>
--- a/vault/50_FGI/FGI 업계/업계섭외현황.xlsx
+++ b/vault/50_FGI/FGI 업계/업계섭외현황.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\뉴프로젝트\2026dgs\vault\02_주요진행상황\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\뉴프로젝트\2026dgs\vault\50_FGI\FGI 업계\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D4DA202-2D97-4E5F-8015-1D59CC32D02F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0C9D8B8-BBF4-4CBA-9751-EA2A288F5C61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27240" yWindow="-255" windowWidth="16860" windowHeight="14970" xr2:uid="{01041B61-266B-4521-86E9-FF95823D999B}"/>
+    <workbookView xWindow="-28920" yWindow="-1605" windowWidth="29040" windowHeight="15840" xr2:uid="{01041B61-266B-4521-86E9-FF95823D999B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="97">
   <si>
     <t>일련
 번호</t>
@@ -1117,7 +1117,9 @@
       <c r="H4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="1"/>
+      <c r="I4" s="1" t="s">
+        <v>93</v>
+      </c>
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
vault backup: 2026-10-19 16:03:06
</commit_message>
<xml_diff>
--- a/vault/50_FGI/FGI 업계/업계섭외현황.xlsx
+++ b/vault/50_FGI/FGI 업계/업계섭외현황.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\뉴프로젝트\2026dgs\vault\50_FGI\FGI 업계\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0C9D8B8-BBF4-4CBA-9751-EA2A288F5C61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8CC28C8-0BA8-4391-98BA-3E3788DBFE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1605" windowWidth="29040" windowHeight="15840" xr2:uid="{01041B61-266B-4521-86E9-FF95823D999B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="118">
   <si>
     <t>일련
 번호</t>
@@ -85,10 +85,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>1차 메일 회신</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>메일 발송 완료</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -409,23 +405,111 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>1차 전화컨택</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>참가의향 메일발송</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>참석 회신</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예정일에 출장</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>황순봉님 휴직 상태임, 출근 안함</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>V 김준겸님 통화, 메일 수신을 못함. ktx7787@daum.net으로 다시 발송함. 연락 취지 전달, 본인이 참석하지 않고 대표가 참석할 것으로 예상, 메일을 확인 후 내일까지 회신하기 함</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>본인 통화, 해당일에 업무로 참석 불가</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>조건부 참석 가능</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>불참 확인</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>대기중</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>메일로 참석 회신, 동반 참석 가능여부에 불가능 회신함</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>메일로 불참 회신</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1차 회신 확인</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>X</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>불참 확인</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>박예은 출장중, 다른 직원 엄수경 님 전화 통화, 공사 참가 요청 메일 내용 알고 있음. 내일까지 참석여부 메일로 회신 주기로 함 --&gt; 엄수경 님 현재 조직개편으로 인한 인력 이동 및 인수인계 시간이라 금번 참석은 어려울 것 같다고 대신 회신</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>V 부재중 3시 이후 다시 통화</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>V 출장 중 오후 4시 이후</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>메일로 참석 회신, 회망일은 12일 (11일, 13일도 무방)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>양미현님은 관광부서에 다른 팀으로 보직 이전, 기존 부서의 김은정 주무관에 안내 메일을 전달하고 업무 이관, 김은정 주무관 통화에서 양미현님 업무를 잘 알지 못한다고 함. 대신해 FGI에 참가는 어렵다고 함</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>V 참가의향은 있으나, 11월 11일만 가능 (11월 12,13일은 출장)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>전화번호가 있는 본원에 있지 않고 분원으로 이전해서 해당 전화반호로 직접 통화 못함. 대신 받은 내부 직원이 전달해 주겠다고 함. 전화번호는 공개하지 않음.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>전화 안받음. 내부 직원도 대신 안받음 -&gt; 대체 전화번호 조사하지 않고 공사에 재확인 요청함</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>전화 연락처 없음 -&gt; 대체 전화번호 조사하지 않고 공사에 재확인 요청함</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>V 02-720-8323 벨 3번 후 팩스 수신음으로 연결됨 -&gt; 승우여행사 대표전화로 걸어서 서신혜님 부재확인(정확한 부재 사유는 이야기하지 않음), 전화받은 담당자가 직접 메일을 확인하고 회신하겠다고 함. -&gt; 메일 내용파악 후 서신혜 (이사)에게 전달하고 내일까지 회신주겠다고 함</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>메일회신 / 전화컨택 내용</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -494,6 +578,40 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="9"/>
+      <color theme="10"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="맑은 고딕"/>
@@ -575,12 +693,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -655,9 +776,37 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1000,8 +1149,8 @@
     <col min="6" max="6" width="12.625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23.125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.125" customWidth="1"/>
-    <col min="10" max="10" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.75" customWidth="1"/>
+    <col min="10" max="10" width="131.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="27" x14ac:dyDescent="0.3">
@@ -1015,25 +1164,25 @@
         <v>1</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>37</v>
-      </c>
       <c r="H1" s="6" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>11</v>
+        <v>104</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -1047,22 +1196,26 @@
         <v>2</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E2" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="G2" s="9" t="s">
-        <v>40</v>
-      </c>
       <c r="H2" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="J2" s="21" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="7">
@@ -1075,22 +1228,26 @@
         <v>2</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E3" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="G3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="G3" s="9" t="s">
-        <v>43</v>
-      </c>
       <c r="H3" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="J3" s="21" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="7">
@@ -1103,24 +1260,26 @@
         <v>2</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E4" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F4" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>45</v>
-      </c>
       <c r="H4" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="J4" s="1"/>
+        <v>106</v>
+      </c>
+      <c r="J4" s="21" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="7">
@@ -1133,22 +1292,26 @@
         <v>3</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E5" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="G5" s="9" t="s">
-        <v>48</v>
-      </c>
       <c r="H5" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="J5" s="21" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="7">
@@ -1161,22 +1324,26 @@
         <v>3</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E6" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="G6" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>51</v>
-      </c>
       <c r="H6" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="J6" s="25" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="7">
@@ -1189,22 +1356,26 @@
         <v>3</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
+        <v>12</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="J7" s="21" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="11">
@@ -1217,22 +1388,26 @@
         <v>4</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="F8" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="G8" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="G8" s="13" t="s">
-        <v>55</v>
-      </c>
       <c r="H8" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="J8" s="22" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="11">
@@ -1245,22 +1420,26 @@
         <v>4</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E9" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F9" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="G9" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="G9" s="13" t="s">
-        <v>58</v>
-      </c>
       <c r="H9" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J9" s="27" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="14">
@@ -1273,22 +1452,26 @@
         <v>4</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E10" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="G10" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="G10" s="13" t="s">
-        <v>61</v>
-      </c>
       <c r="H10" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="I10" s="28" t="s">
+        <v>99</v>
+      </c>
+      <c r="J10" s="22" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="11">
@@ -1301,22 +1484,26 @@
         <v>4</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E11" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="F11" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F11" s="12" t="s">
+      <c r="G11" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="G11" s="13" t="s">
-        <v>64</v>
-      </c>
       <c r="H11" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J11" s="27" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="11">
@@ -1329,22 +1516,26 @@
         <v>4</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E12" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F12" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="G12" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="G12" s="12" t="s">
-        <v>67</v>
-      </c>
       <c r="H12" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="J12" s="22" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="11">
@@ -1357,24 +1548,26 @@
         <v>5</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E13" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F13" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="G13" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="G13" s="13" t="s">
-        <v>70</v>
-      </c>
       <c r="H13" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="J13" s="2"/>
+        <v>92</v>
+      </c>
+      <c r="J13" s="22" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="14">
@@ -1387,24 +1580,26 @@
         <v>5</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E14" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="G14" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="G14" s="13" t="s">
-        <v>73</v>
-      </c>
       <c r="H14" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="J14" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="I14" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="J14" s="22" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="11">
@@ -1417,25 +1612,25 @@
         <v>5</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E15" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="F15" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="G15" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="G15" s="13" t="s">
-        <v>76</v>
-      </c>
       <c r="H15" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>42</v>
+        <v>92</v>
+      </c>
+      <c r="J15" s="22" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
@@ -1449,22 +1644,26 @@
         <v>5</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
+        <v>12</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="J16" s="22" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="11">
@@ -1477,22 +1676,26 @@
         <v>5</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E17" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="G17" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="G17" s="13" t="s">
-        <v>80</v>
-      </c>
       <c r="H17" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J17" s="22" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="18">
@@ -1505,24 +1708,26 @@
         <v>6</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E18" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="F18" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="19" t="s">
+      <c r="G18" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="G18" s="20" t="s">
-        <v>83</v>
-      </c>
       <c r="H18" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="J18" s="3"/>
+        <v>11</v>
+      </c>
+      <c r="I18" s="29" t="s">
+        <v>94</v>
+      </c>
+      <c r="J18" s="23" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="18">
@@ -1535,22 +1740,26 @@
         <v>6</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E19" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="F19" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="F19" s="19" t="s">
+      <c r="G19" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="G19" s="20" t="s">
-        <v>86</v>
-      </c>
       <c r="H19" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
+        <v>11</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J19" s="23" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="18">
@@ -1563,22 +1772,26 @@
         <v>6</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E20" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="F20" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="F20" s="19" t="s">
+      <c r="G20" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="G20" s="20" t="s">
-        <v>89</v>
-      </c>
       <c r="H20" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
+        <v>11</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="J20" s="23" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="18">
@@ -1591,22 +1804,26 @@
         <v>6</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E21" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="F21" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="F21" s="19" t="s">
+      <c r="G21" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="G21" s="20" t="s">
-        <v>92</v>
-      </c>
       <c r="H21" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
+        <v>11</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J21" s="23" t="s">
+        <v>114</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1616,6 +1833,10 @@
       <formula2>99999999</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="G6" r:id="rId1" xr:uid="{4DA085C7-430A-49E9-AD57-66340464A825}"/>
+    <hyperlink ref="G5" r:id="rId2" xr:uid="{9864FBCA-94E4-4BD8-9CA4-C9F408390D70}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-10-19 16:55:25
</commit_message>
<xml_diff>
--- a/vault/50_FGI/FGI 업계/업계섭외현황.xlsx
+++ b/vault/50_FGI/FGI 업계/업계섭외현황.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\뉴프로젝트\2026dgs\vault\50_FGI\FGI 업계\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB89BB58-182F-453D-B8C6-60CB23DC3548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65068C70-544E-45CD-983C-D4AD8D5B52E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1605" windowWidth="29040" windowHeight="15840" tabRatio="333" xr2:uid="{01041B61-266B-4521-86E9-FF95823D999B}"/>
   </bookViews>
@@ -413,6 +413,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>조건부 참석 가능</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>불참 확인</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -437,10 +441,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>전화 안받음. 내부 직원도 대신 안받음 -&gt; 대체 전화번호 조사하지 않고 공사에 재확인 요청함</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>메일회신 / 전화컨택 내용</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -449,10 +449,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>전화 연락처 없음 -&gt; 전화번호 조사하지 않고 공사에 확인 요청함</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>회신대기중</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -502,14 +498,6 @@
   </si>
   <si>
     <t>참석</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>연락처없음 / 전화안됨 5</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>조건부 참석</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -535,6 +523,18 @@
   </si>
   <si>
     <t>부재중 3시 이후 다시 통화 -&gt; 직접 통화됨, 좀더 고민하고 메일로 회신주기로 함 -&gt; 메일로 참석 회신함 11일, 13일 추천, 12일도 가능함</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>전화 안받음 -&gt; 김려경 님 통화됨 -&gt; 일정 확인 후 메일로 회신하기로 함</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>전화 안받음 -&gt; 전화 안받음</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>연락처없음 / 전화안됨 4</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -684,12 +684,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFD6D6D6"/>
       </patternFill>
@@ -703,6 +697,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -746,16 +746,13 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -794,20 +791,9 @@
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -817,13 +803,10 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -836,9 +819,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -857,11 +837,31 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1206,726 +1206,726 @@
     <col min="4" max="4" width="18.625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21" style="24" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" style="19" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.375" customWidth="1"/>
-    <col min="10" max="10" width="69.5" style="31" customWidth="1"/>
+    <col min="10" max="10" width="69.5" style="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="26.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
-        <v>122</v>
-      </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
+      <c r="A1" s="26" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
     </row>
     <row r="2" spans="1:10" ht="26.25" x14ac:dyDescent="0.3">
-      <c r="A2" s="33"/>
-      <c r="B2" s="36" t="s">
-        <v>117</v>
-      </c>
-      <c r="C2" s="37">
+      <c r="A2" s="27"/>
+      <c r="B2" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2" s="31">
         <v>3</v>
       </c>
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="E2" s="31">
+        <v>2</v>
+      </c>
+      <c r="F2" s="30" t="s">
         <v>115</v>
       </c>
-      <c r="E2" s="37">
-        <v>2</v>
-      </c>
-      <c r="F2" s="36" t="s">
-        <v>116</v>
-      </c>
-      <c r="G2" s="37">
+      <c r="G2" s="31">
         <v>7</v>
       </c>
-      <c r="H2" s="36" t="s">
-        <v>105</v>
-      </c>
-      <c r="I2" s="37">
-        <v>3</v>
-      </c>
-      <c r="J2" s="36" t="s">
-        <v>118</v>
+      <c r="H2" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="I2" s="31">
+        <v>4</v>
+      </c>
+      <c r="J2" s="30" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="B5" s="6" t="s">
+      <c r="A5" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="I5" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="J5" s="25" t="s">
+      <c r="I5" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="J5" s="20" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="36" x14ac:dyDescent="0.3">
-      <c r="A6" s="7">
+      <c r="A6" s="6">
         <v>9</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G6" s="21" t="s">
+      <c r="G6" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="6" t="s">
         <v>10</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="J6" s="26" t="s">
-        <v>120</v>
+      <c r="J6" s="21" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="7">
+      <c r="A7" s="6">
         <v>10</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="G7" s="21" t="s">
+      <c r="G7" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="6" t="s">
         <v>10</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="J7" s="26" t="s">
-        <v>104</v>
+        <v>98</v>
+      </c>
+      <c r="J7" s="21" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="7">
+      <c r="A8" s="6">
         <v>11</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="G8" s="21" t="s">
+      <c r="G8" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="6" t="s">
         <v>10</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="J8" s="26" t="s">
-        <v>123</v>
+        <v>99</v>
+      </c>
+      <c r="J8" s="21" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="36" x14ac:dyDescent="0.3">
-      <c r="A9" s="7">
+      <c r="A9" s="6">
         <v>12</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="F9" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="G9" s="21" t="s">
+      <c r="F9" s="28" t="s">
+        <v>118</v>
+      </c>
+      <c r="G9" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="I9" s="20" t="s">
-        <v>119</v>
-      </c>
-      <c r="J9" s="27" t="s">
-        <v>106</v>
+      <c r="I9" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="J9" s="22" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="24" x14ac:dyDescent="0.3">
-      <c r="A10" s="7">
+      <c r="A10" s="6">
         <v>13</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="G10" s="21" t="s">
+      <c r="G10" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="6" t="s">
         <v>10</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="J10" s="35" t="s">
+      <c r="J10" s="29" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="7">
+      <c r="A11" s="6">
         <v>14</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="8" t="s">
         <v>11</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="J11" s="26" t="s">
+        <v>98</v>
+      </c>
+      <c r="J11" s="21" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="10">
+      <c r="A12" s="9">
         <v>3</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="22" t="s">
+      <c r="G12" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="9" t="s">
         <v>10</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="J12" s="28" t="s">
-        <v>107</v>
+        <v>96</v>
+      </c>
+      <c r="J12" s="23" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="24" x14ac:dyDescent="0.3">
-      <c r="A13" s="10">
+      <c r="A13" s="9">
         <v>4</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="G13" s="22" t="s">
+      <c r="G13" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="I13" s="18" t="s">
+      <c r="I13" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="J13" s="29" t="s">
-        <v>125</v>
+      <c r="J13" s="24" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="12">
+      <c r="A14" s="11">
         <v>5</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="G14" s="22" t="s">
+      <c r="G14" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="H14" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="I14" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="J14" s="28" t="s">
-        <v>108</v>
+      <c r="I14" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="J14" s="23" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="24" x14ac:dyDescent="0.3">
-      <c r="A15" s="10">
+      <c r="A15" s="9">
         <v>8</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="G15" s="22" t="s">
+      <c r="G15" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="H15" s="10" t="s">
+      <c r="H15" s="9" t="s">
         <v>10</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="J15" s="29" t="s">
-        <v>124</v>
+        <v>104</v>
+      </c>
+      <c r="J15" s="24" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="36" x14ac:dyDescent="0.3">
-      <c r="A16" s="10">
+      <c r="A16" s="9">
         <v>20</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="13" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="F16" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="H16" s="14" t="s">
+      <c r="H16" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="J16" s="28" t="s">
-        <v>100</v>
+        <v>96</v>
+      </c>
+      <c r="J16" s="23" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="10">
+      <c r="A17" s="9">
         <v>6</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="F17" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="G17" s="22" t="s">
+      <c r="G17" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="H17" s="9" t="s">
         <v>10</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="J17" s="28" t="s">
-        <v>109</v>
+      <c r="J17" s="23" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="12">
+      <c r="A18" s="11">
         <v>7</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="F18" s="13" t="s">
+      <c r="F18" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G18" s="22" t="s">
+      <c r="G18" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="H18" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="I18" s="18" t="s">
+      <c r="I18" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="J18" s="28" t="s">
-        <v>99</v>
+      <c r="J18" s="23" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="10">
+      <c r="A19" s="9">
         <v>16</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="G19" s="22" t="s">
+      <c r="G19" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="H19" s="9" t="s">
         <v>10</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="J19" s="28" t="s">
-        <v>110</v>
+      <c r="J19" s="23" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="10">
+      <c r="A20" s="9">
         <v>17</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F20" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G20" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="H20" s="15" t="s">
+      <c r="H20" s="14" t="s">
         <v>11</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="J20" s="28" t="s">
+        <v>98</v>
+      </c>
+      <c r="J20" s="23" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="24" x14ac:dyDescent="0.3">
-      <c r="A21" s="10">
+      <c r="A21" s="9">
         <v>19</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="13" t="s">
         <v>8</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="11" t="s">
+      <c r="E21" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="F21" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="G21" s="22" t="s">
+      <c r="G21" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="H21" s="14" t="s">
+      <c r="H21" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="J21" s="28" t="s">
+        <v>104</v>
+      </c>
+      <c r="J21" s="23" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A22" s="32">
+        <v>1</v>
+      </c>
+      <c r="B22" s="32" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="33" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="E22" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="F22" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="G22" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="H22" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="I22" s="36" t="s">
+        <v>92</v>
+      </c>
+      <c r="J22" s="37" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="16">
-        <v>1</v>
-      </c>
-      <c r="B22" s="16" t="s">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A23" s="32">
+        <v>2</v>
+      </c>
+      <c r="B23" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C23" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="E22" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="F22" s="17" t="s">
-        <v>79</v>
-      </c>
-      <c r="G22" s="23" t="s">
-        <v>80</v>
-      </c>
-      <c r="H22" s="16" t="s">
+      <c r="D23" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="E23" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="F23" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="G23" s="35" t="s">
+        <v>83</v>
+      </c>
+      <c r="H23" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="I22" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="J22" s="30" t="s">
+      <c r="I23" s="33" t="s">
+        <v>104</v>
+      </c>
+      <c r="J23" s="37" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="32">
+        <v>15</v>
+      </c>
+      <c r="B24" s="32" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="33" t="s">
+        <v>5</v>
+      </c>
+      <c r="D24" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="E24" s="34" t="s">
+        <v>84</v>
+      </c>
+      <c r="F24" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="G24" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="H24" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="I24" s="33" t="s">
+        <v>99</v>
+      </c>
+      <c r="J24" s="37" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="16">
-        <v>2</v>
-      </c>
-      <c r="B23" s="16" t="s">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="32">
+        <v>18</v>
+      </c>
+      <c r="B25" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C25" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="D23" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E23" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="F23" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="G23" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="H23" s="16" t="s">
+      <c r="D25" s="34" t="s">
+        <v>32</v>
+      </c>
+      <c r="E25" s="34" t="s">
+        <v>87</v>
+      </c>
+      <c r="F25" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="G25" s="35" t="s">
+        <v>89</v>
+      </c>
+      <c r="H25" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="I23" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="J23" s="30" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="16">
-        <v>15</v>
-      </c>
-      <c r="B24" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="E24" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="F24" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="G24" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="H24" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I24" s="3" t="s">
+      <c r="I25" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="J24" s="30" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="16">
-        <v>18</v>
-      </c>
-      <c r="B25" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D25" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="E25" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="F25" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="G25" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="H25" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I25" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="J25" s="30" t="s">
-        <v>101</v>
+      <c r="J25" s="37" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>